<commit_message>
MCA and Btech TR Excel Modifed
</commit_message>
<xml_diff>
--- a/mca_sem/static/TR/MCA_1_TR_FORMATE.xlsx
+++ b/mca_sem/static/TR/MCA_1_TR_FORMATE.xlsx
@@ -167,7 +167,7 @@
     <t>2418M240007</t>
   </si>
   <si>
-    <t>No. of Candidate:  05</t>
+    <t>No. of Students:  05</t>
   </si>
   <si>
     <t>First Class with Distinction:</t>
@@ -209,7 +209,7 @@
     <t xml:space="preserve">Address </t>
   </si>
   <si>
-    <t>Qualified: 04</t>
+    <t>Qualified:</t>
   </si>
   <si>
     <t>Pass: 04</t>
@@ -1778,7 +1778,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1" spans="1:29">
+    <row r="8" ht="61" customHeight="1" spans="1:29">
       <c r="A8" s="12" t="s">
         <v>17</v>
       </c>

</xml_diff>